<commit_message>
Update processed jobs state
</commit_message>
<xml_diff>
--- a/job_tracker.xlsx
+++ b/job_tracker.xlsx
@@ -103,7 +103,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="60">
+  <cellXfs count="61">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -269,6 +269,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -645,7 +648,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K61"/>
+  <dimension ref="A1:K63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -719,12 +722,12 @@
       </c>
     </row>
     <row r="2" ht="18" customHeight="1">
-      <c r="A2" s="58" t="inlineStr">
-        <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="B2" s="58" t="inlineStr">
+      <c r="A2" s="60" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B2" s="60" t="inlineStr">
         <is>
           <t>4433259032</t>
         </is>
@@ -749,7 +752,7 @@
           <t>https://www.linkedin.com/jobs/view/junior-full-stack-web-developer-at-open-healthcare-4433259032</t>
         </is>
       </c>
-      <c r="G2" s="58" t="inlineStr">
+      <c r="G2" s="60" t="inlineStr">
         <is>
           <t>95%</t>
         </is>
@@ -764,24 +767,24 @@
           <t>resume_Junior_Full-Stack_Web_Develope_OPEN_Healthcare_131200.docx</t>
         </is>
       </c>
-      <c r="J2" s="58" t="inlineStr">
-        <is>
-          <t>No (Base)</t>
-        </is>
-      </c>
-      <c r="K2" s="58" t="inlineStr">
+      <c r="J2" s="60" t="inlineStr">
+        <is>
+          <t>No (Base)</t>
+        </is>
+      </c>
+      <c r="K2" s="60" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
       </c>
     </row>
     <row r="3" ht="18" customHeight="1">
-      <c r="A3" s="58" t="inlineStr">
-        <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="B3" s="58" t="inlineStr">
+      <c r="A3" s="60" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B3" s="60" t="inlineStr">
         <is>
           <t>4432623804</t>
         </is>
@@ -806,7 +809,7 @@
           <t>https://sa.linkedin.com/jobs/view/full-stack-developer-at-emdad-by-elm-4432623804</t>
         </is>
       </c>
-      <c r="G3" s="58" t="inlineStr">
+      <c r="G3" s="60" t="inlineStr">
         <is>
           <t>95%</t>
         </is>
@@ -821,24 +824,24 @@
           <t>resume_Full_Stack_Developer_Emdad_By_Elm_131211.docx</t>
         </is>
       </c>
-      <c r="J3" s="58" t="inlineStr">
-        <is>
-          <t>No (Base)</t>
-        </is>
-      </c>
-      <c r="K3" s="58" t="inlineStr">
+      <c r="J3" s="60" t="inlineStr">
+        <is>
+          <t>No (Base)</t>
+        </is>
+      </c>
+      <c r="K3" s="60" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
       </c>
     </row>
     <row r="4" ht="18" customHeight="1">
-      <c r="A4" s="58" t="inlineStr">
-        <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="B4" s="58" t="inlineStr">
+      <c r="A4" s="60" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B4" s="60" t="inlineStr">
         <is>
           <t>4433653887</t>
         </is>
@@ -863,7 +866,7 @@
           <t>https://www.linkedin.com/jobs/view/full-stack-web-developer-at-lynkup-4433653887</t>
         </is>
       </c>
-      <c r="G4" s="58" t="inlineStr">
+      <c r="G4" s="60" t="inlineStr">
         <is>
           <t>95%</t>
         </is>
@@ -878,24 +881,24 @@
           <t>resume_Full_Stack_Web_Developer_LYNKUP_131220.docx</t>
         </is>
       </c>
-      <c r="J4" s="58" t="inlineStr">
-        <is>
-          <t>No (Base)</t>
-        </is>
-      </c>
-      <c r="K4" s="58" t="inlineStr">
+      <c r="J4" s="60" t="inlineStr">
+        <is>
+          <t>No (Base)</t>
+        </is>
+      </c>
+      <c r="K4" s="60" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
       </c>
     </row>
     <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="58" t="inlineStr">
-        <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="B5" s="58" t="inlineStr">
+      <c r="A5" s="60" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B5" s="60" t="inlineStr">
         <is>
           <t>4434428780</t>
         </is>
@@ -920,7 +923,7 @@
           <t>https://de.linkedin.com/jobs/view/freelance-full-stack-web-app-developer-at-mindrift-4434428780</t>
         </is>
       </c>
-      <c r="G5" s="58" t="inlineStr">
+      <c r="G5" s="60" t="inlineStr">
         <is>
           <t>95%</t>
         </is>
@@ -935,24 +938,24 @@
           <t>resume_Freelance_Full-Stack_Web_App_D_Mindrift_131230.docx</t>
         </is>
       </c>
-      <c r="J5" s="58" t="inlineStr">
-        <is>
-          <t>No (Base)</t>
-        </is>
-      </c>
-      <c r="K5" s="58" t="inlineStr">
+      <c r="J5" s="60" t="inlineStr">
+        <is>
+          <t>No (Base)</t>
+        </is>
+      </c>
+      <c r="K5" s="60" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
       </c>
     </row>
     <row r="6" ht="18" customHeight="1">
-      <c r="A6" s="58" t="inlineStr">
-        <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="B6" s="58" t="inlineStr">
+      <c r="A6" s="60" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B6" s="60" t="inlineStr">
         <is>
           <t>4434439187</t>
         </is>
@@ -977,7 +980,7 @@
           <t>https://ie.linkedin.com/jobs/view/freelance-full-stack-web-app-developer-at-mindrift-4434439187</t>
         </is>
       </c>
-      <c r="G6" s="58" t="inlineStr">
+      <c r="G6" s="60" t="inlineStr">
         <is>
           <t>95%</t>
         </is>
@@ -992,12 +995,12 @@
           <t>resume_Freelance_Full-Stack_Web_App_D_Mindrift_131241.docx</t>
         </is>
       </c>
-      <c r="J6" s="58" t="inlineStr">
-        <is>
-          <t>No (Base)</t>
-        </is>
-      </c>
-      <c r="K6" s="58" t="inlineStr">
+      <c r="J6" s="60" t="inlineStr">
+        <is>
+          <t>No (Base)</t>
+        </is>
+      </c>
+      <c r="K6" s="60" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
@@ -1118,12 +1121,12 @@
       </c>
     </row>
     <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="58" t="inlineStr">
-        <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="B9" s="58" t="inlineStr">
+      <c r="A9" s="60" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B9" s="60" t="inlineStr">
         <is>
           <t>4434085791</t>
         </is>
@@ -1148,7 +1151,7 @@
           <t>https://sa.linkedin.com/jobs/view/junior-front-end-developer-remote-at-pulsemedia-emea-4434085791</t>
         </is>
       </c>
-      <c r="G9" s="58" t="inlineStr">
+      <c r="G9" s="60" t="inlineStr">
         <is>
           <t>95%</t>
         </is>
@@ -1163,24 +1166,24 @@
           <t>resume_Junior_Front-End_Developer_Rem_PULSEMEDIA_EMEA_131311.docx</t>
         </is>
       </c>
-      <c r="J9" s="58" t="inlineStr">
-        <is>
-          <t>No (Base)</t>
-        </is>
-      </c>
-      <c r="K9" s="58" t="inlineStr">
+      <c r="J9" s="60" t="inlineStr">
+        <is>
+          <t>No (Base)</t>
+        </is>
+      </c>
+      <c r="K9" s="60" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
       </c>
     </row>
     <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="58" t="inlineStr">
-        <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="B10" s="58" t="inlineStr">
+      <c r="A10" s="60" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B10" s="60" t="inlineStr">
         <is>
           <t>4434256892</t>
         </is>
@@ -1205,7 +1208,7 @@
           <t>https://sa.linkedin.com/jobs/view/junior-front-end-developer-remote-at-pulsemedia-emea-4434256892</t>
         </is>
       </c>
-      <c r="G10" s="58" t="inlineStr">
+      <c r="G10" s="60" t="inlineStr">
         <is>
           <t>95%</t>
         </is>
@@ -1220,24 +1223,24 @@
           <t>resume_Junior_Front-End_Developer_Rem_PULSEMEDIA_EMEA_131320.docx</t>
         </is>
       </c>
-      <c r="J10" s="58" t="inlineStr">
-        <is>
-          <t>No (Base)</t>
-        </is>
-      </c>
-      <c r="K10" s="58" t="inlineStr">
+      <c r="J10" s="60" t="inlineStr">
+        <is>
+          <t>No (Base)</t>
+        </is>
+      </c>
+      <c r="K10" s="60" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="58" t="inlineStr">
-        <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="B11" s="58" t="inlineStr">
+      <c r="A11" s="60" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B11" s="60" t="inlineStr">
         <is>
           <t>4434078864</t>
         </is>
@@ -1262,7 +1265,7 @@
           <t>https://sa.linkedin.com/jobs/view/junior-front-end-developer-remote-at-pulsemedia-emea-4434078864</t>
         </is>
       </c>
-      <c r="G11" s="58" t="inlineStr">
+      <c r="G11" s="60" t="inlineStr">
         <is>
           <t>90%</t>
         </is>
@@ -1277,24 +1280,24 @@
           <t>resume_Junior_Front-End_Developer_Rem_PULSEMEDIA_EMEA_131330.docx</t>
         </is>
       </c>
-      <c r="J11" s="58" t="inlineStr">
-        <is>
-          <t>No (Base)</t>
-        </is>
-      </c>
-      <c r="K11" s="58" t="inlineStr">
+      <c r="J11" s="60" t="inlineStr">
+        <is>
+          <t>No (Base)</t>
+        </is>
+      </c>
+      <c r="K11" s="60" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
       </c>
     </row>
     <row r="12" ht="18" customHeight="1">
-      <c r="A12" s="58" t="inlineStr">
-        <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="B12" s="58" t="inlineStr">
+      <c r="A12" s="60" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B12" s="60" t="inlineStr">
         <is>
           <t>4433237709</t>
         </is>
@@ -1319,7 +1322,7 @@
           <t>https://www.linkedin.com/jobs/view/junior-full-stack-web-developer-at-fortray-global-service-limited-4433237709</t>
         </is>
       </c>
-      <c r="G12" s="58" t="inlineStr">
+      <c r="G12" s="60" t="inlineStr">
         <is>
           <t>95%</t>
         </is>
@@ -1334,24 +1337,24 @@
           <t>resume_Junior_Full_Stack_Web_Develope_Fortray_Global_Ser_132112.docx</t>
         </is>
       </c>
-      <c r="J12" s="58" t="inlineStr">
-        <is>
-          <t>No (Base)</t>
-        </is>
-      </c>
-      <c r="K12" s="58" t="inlineStr">
+      <c r="J12" s="60" t="inlineStr">
+        <is>
+          <t>No (Base)</t>
+        </is>
+      </c>
+      <c r="K12" s="60" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
       </c>
     </row>
     <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="58" t="inlineStr">
-        <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="B13" s="58" t="inlineStr">
+      <c r="A13" s="60" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B13" s="60" t="inlineStr">
         <is>
           <t>4431074962</t>
         </is>
@@ -1376,7 +1379,7 @@
           <t>https://in.linkedin.com/jobs/view/mern-stack-developer-at-kba-systems-4431074962</t>
         </is>
       </c>
-      <c r="G13" s="58" t="inlineStr">
+      <c r="G13" s="60" t="inlineStr">
         <is>
           <t>100%</t>
         </is>
@@ -1391,24 +1394,24 @@
           <t>resume_MERN_Stack_Developer_KBA_Systems_132125.docx</t>
         </is>
       </c>
-      <c r="J13" s="58" t="inlineStr">
-        <is>
-          <t>No (Base)</t>
-        </is>
-      </c>
-      <c r="K13" s="58" t="inlineStr">
+      <c r="J13" s="60" t="inlineStr">
+        <is>
+          <t>No (Base)</t>
+        </is>
+      </c>
+      <c r="K13" s="60" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
       </c>
     </row>
     <row r="14" ht="18" customHeight="1">
-      <c r="A14" s="58" t="inlineStr">
-        <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="B14" s="58" t="inlineStr">
+      <c r="A14" s="60" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B14" s="60" t="inlineStr">
         <is>
           <t>4433570601</t>
         </is>
@@ -1433,7 +1436,7 @@
           <t>https://in.linkedin.com/jobs/view/full-stack-developer-at-uest-4433570601</t>
         </is>
       </c>
-      <c r="G14" s="58" t="inlineStr">
+      <c r="G14" s="60" t="inlineStr">
         <is>
           <t>95%</t>
         </is>
@@ -1448,24 +1451,24 @@
           <t>resume_Full_Stack_Developer_Uest_132136.docx</t>
         </is>
       </c>
-      <c r="J14" s="58" t="inlineStr">
-        <is>
-          <t>No (Base)</t>
-        </is>
-      </c>
-      <c r="K14" s="58" t="inlineStr">
+      <c r="J14" s="60" t="inlineStr">
+        <is>
+          <t>No (Base)</t>
+        </is>
+      </c>
+      <c r="K14" s="60" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1">
-      <c r="A15" s="58" t="inlineStr">
-        <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="B15" s="58" t="inlineStr">
+      <c r="A15" s="60" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B15" s="60" t="inlineStr">
         <is>
           <t>4431848139</t>
         </is>
@@ -1490,7 +1493,7 @@
           <t>https://in.linkedin.com/jobs/view/software-engineer-at-plexus-digitals-pvt-ltd-4431848139</t>
         </is>
       </c>
-      <c r="G15" s="58" t="inlineStr">
+      <c r="G15" s="60" t="inlineStr">
         <is>
           <t>95%</t>
         </is>
@@ -1505,12 +1508,12 @@
           <t>resume_Software_Engineer_Plexus_Digitals_Pv_132150.docx</t>
         </is>
       </c>
-      <c r="J15" s="58" t="inlineStr">
-        <is>
-          <t>No (Base)</t>
-        </is>
-      </c>
-      <c r="K15" s="58" t="inlineStr">
+      <c r="J15" s="60" t="inlineStr">
+        <is>
+          <t>No (Base)</t>
+        </is>
+      </c>
+      <c r="K15" s="60" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
@@ -1588,12 +1591,12 @@
       </c>
     </row>
     <row r="19" ht="18" customHeight="1">
-      <c r="A19" s="58" t="inlineStr">
-        <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="B19" s="58" t="inlineStr">
+      <c r="A19" s="60" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B19" s="60" t="inlineStr">
         <is>
           <t>4433647089</t>
         </is>
@@ -1618,7 +1621,7 @@
           <t>https://au.linkedin.com/jobs/view/web-application-developer-at-senso-cloud-%E2%9A%A1-4433647089</t>
         </is>
       </c>
-      <c r="G19" s="58" t="inlineStr">
+      <c r="G19" s="60" t="inlineStr">
         <is>
           <t>95%</t>
         </is>
@@ -1633,24 +1636,24 @@
           <t>resume_Web_Application_Developer_sensocloud_132627.docx</t>
         </is>
       </c>
-      <c r="J19" s="58" t="inlineStr">
-        <is>
-          <t>No (Base)</t>
-        </is>
-      </c>
-      <c r="K19" s="58" t="inlineStr">
+      <c r="J19" s="60" t="inlineStr">
+        <is>
+          <t>No (Base)</t>
+        </is>
+      </c>
+      <c r="K19" s="60" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
-      <c r="A20" s="58" t="inlineStr">
-        <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="B20" s="58" t="inlineStr">
+      <c r="A20" s="60" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B20" s="60" t="inlineStr">
         <is>
           <t>4433594140</t>
         </is>
@@ -1675,7 +1678,7 @@
           <t>https://au.linkedin.com/jobs/view/full-stack-developer-at-qantas-4433594140</t>
         </is>
       </c>
-      <c r="G20" s="58" t="inlineStr">
+      <c r="G20" s="60" t="inlineStr">
         <is>
           <t>90%</t>
         </is>
@@ -1690,12 +1693,12 @@
           <t>resume_Full_Stack_Developer_Qantas_132640.docx</t>
         </is>
       </c>
-      <c r="J20" s="58" t="inlineStr">
-        <is>
-          <t>No (Base)</t>
-        </is>
-      </c>
-      <c r="K20" s="58" t="inlineStr">
+      <c r="J20" s="60" t="inlineStr">
+        <is>
+          <t>No (Base)</t>
+        </is>
+      </c>
+      <c r="K20" s="60" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
@@ -1759,12 +1762,12 @@
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
-      <c r="A22" s="58" t="inlineStr">
-        <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="B22" s="58" t="inlineStr">
+      <c r="A22" s="60" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B22" s="60" t="inlineStr">
         <is>
           <t>4429402964</t>
         </is>
@@ -1789,7 +1792,7 @@
           <t>https://au.linkedin.com/jobs/view/software-engineer-at-workyard-4429402964</t>
         </is>
       </c>
-      <c r="G22" s="58" t="inlineStr">
+      <c r="G22" s="60" t="inlineStr">
         <is>
           <t>95%</t>
         </is>
@@ -1804,24 +1807,24 @@
           <t>resume_Software_Engineer_Workyard_132707.docx</t>
         </is>
       </c>
-      <c r="J22" s="58" t="inlineStr">
-        <is>
-          <t>No (Base)</t>
-        </is>
-      </c>
-      <c r="K22" s="58" t="inlineStr">
+      <c r="J22" s="60" t="inlineStr">
+        <is>
+          <t>No (Base)</t>
+        </is>
+      </c>
+      <c r="K22" s="60" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
-      <c r="A23" s="58" t="inlineStr">
-        <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="B23" s="58" t="inlineStr">
+      <c r="A23" s="60" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B23" s="60" t="inlineStr">
         <is>
           <t>4434416638</t>
         </is>
@@ -1846,7 +1849,7 @@
           <t>https://sa.linkedin.com/jobs/view/junior-front-end-developer-remote-at-pulsemedia-emea-4434416638</t>
         </is>
       </c>
-      <c r="G23" s="58" t="inlineStr">
+      <c r="G23" s="60" t="inlineStr">
         <is>
           <t>90%</t>
         </is>
@@ -1861,24 +1864,24 @@
           <t>resume_Junior_Front-End_Developer_Rem_PULSEMEDIA_EMEA_132718.docx</t>
         </is>
       </c>
-      <c r="J23" s="58" t="inlineStr">
-        <is>
-          <t>No (Base)</t>
-        </is>
-      </c>
-      <c r="K23" s="58" t="inlineStr">
+      <c r="J23" s="60" t="inlineStr">
+        <is>
+          <t>No (Base)</t>
+        </is>
+      </c>
+      <c r="K23" s="60" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
-      <c r="A24" s="58" t="inlineStr">
-        <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="B24" s="58" t="inlineStr">
+      <c r="A24" s="60" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B24" s="60" t="inlineStr">
         <is>
           <t>4434458375</t>
         </is>
@@ -1903,7 +1906,7 @@
           <t>https://eg.linkedin.com/jobs/view/internship-%E2%80%93-full-stack-developer-mern-nestjs-at-awfar-com-4434458375</t>
         </is>
       </c>
-      <c r="G24" s="58" t="inlineStr">
+      <c r="G24" s="60" t="inlineStr">
         <is>
           <t>95%</t>
         </is>
@@ -1918,24 +1921,24 @@
           <t>resume_Internship__Full_Stack_Develop_Awfarcom_132729.docx</t>
         </is>
       </c>
-      <c r="J24" s="58" t="inlineStr">
-        <is>
-          <t>No (Base)</t>
-        </is>
-      </c>
-      <c r="K24" s="58" t="inlineStr">
+      <c r="J24" s="60" t="inlineStr">
+        <is>
+          <t>No (Base)</t>
+        </is>
+      </c>
+      <c r="K24" s="60" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
-      <c r="A25" s="58" t="inlineStr">
-        <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="B25" s="58" t="inlineStr">
+      <c r="A25" s="60" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B25" s="60" t="inlineStr">
         <is>
           <t>4433815246</t>
         </is>
@@ -1960,7 +1963,7 @@
           <t>https://ch.linkedin.com/jobs/view/full-stack-developer-mern-stack-fully-remote-at-zytech-digital-solutions-4433815246</t>
         </is>
       </c>
-      <c r="G25" s="58" t="inlineStr">
+      <c r="G25" s="60" t="inlineStr">
         <is>
           <t>100%</t>
         </is>
@@ -1975,24 +1978,24 @@
           <t>resume_Full_Stack_Developer_MERN_Stac_Zytech_Digital_Sol_132739.docx</t>
         </is>
       </c>
-      <c r="J25" s="58" t="inlineStr">
-        <is>
-          <t>No (Base)</t>
-        </is>
-      </c>
-      <c r="K25" s="58" t="inlineStr">
+      <c r="J25" s="60" t="inlineStr">
+        <is>
+          <t>No (Base)</t>
+        </is>
+      </c>
+      <c r="K25" s="60" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
       </c>
     </row>
     <row r="26" ht="18" customHeight="1">
-      <c r="A26" s="58" t="inlineStr">
-        <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="B26" s="58" t="inlineStr">
+      <c r="A26" s="60" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B26" s="60" t="inlineStr">
         <is>
           <t>4432541944</t>
         </is>
@@ -2017,7 +2020,7 @@
           <t>https://in.linkedin.com/jobs/view/full-stack-developer-mern-at-comviva-4432541944</t>
         </is>
       </c>
-      <c r="G26" s="58" t="inlineStr">
+      <c r="G26" s="60" t="inlineStr">
         <is>
           <t>100%</t>
         </is>
@@ -2032,24 +2035,24 @@
           <t>resume_Full_Stack_Developer_MERN_Comviva_132751.docx</t>
         </is>
       </c>
-      <c r="J26" s="58" t="inlineStr">
-        <is>
-          <t>No (Base)</t>
-        </is>
-      </c>
-      <c r="K26" s="58" t="inlineStr">
+      <c r="J26" s="60" t="inlineStr">
+        <is>
+          <t>No (Base)</t>
+        </is>
+      </c>
+      <c r="K26" s="60" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
       </c>
     </row>
     <row r="27" ht="18" customHeight="1">
-      <c r="A27" s="58" t="inlineStr">
-        <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="B27" s="58" t="inlineStr">
+      <c r="A27" s="60" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B27" s="60" t="inlineStr">
         <is>
           <t>4431092395</t>
         </is>
@@ -2074,7 +2077,7 @@
           <t>https://in.linkedin.com/jobs/view/full-stack-developer-intern-at-yathi-solutions-4431092395</t>
         </is>
       </c>
-      <c r="G27" s="58" t="inlineStr">
+      <c r="G27" s="60" t="inlineStr">
         <is>
           <t>95%</t>
         </is>
@@ -2089,24 +2092,24 @@
           <t>resume_Full_Stack_Developer_Intern_Yathi_Solutions_132803.docx</t>
         </is>
       </c>
-      <c r="J27" s="58" t="inlineStr">
-        <is>
-          <t>No (Base)</t>
-        </is>
-      </c>
-      <c r="K27" s="58" t="inlineStr">
+      <c r="J27" s="60" t="inlineStr">
+        <is>
+          <t>No (Base)</t>
+        </is>
+      </c>
+      <c r="K27" s="60" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
-      <c r="A28" s="58" t="inlineStr">
-        <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="B28" s="58" t="inlineStr">
+      <c r="A28" s="60" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B28" s="60" t="inlineStr">
         <is>
           <t>4333363253</t>
         </is>
@@ -2131,7 +2134,7 @@
           <t>https://in.linkedin.com/jobs/view/staff-engineer-full-stack-mern-at-forbes-advisor-4333363253</t>
         </is>
       </c>
-      <c r="G28" s="58" t="inlineStr">
+      <c r="G28" s="60" t="inlineStr">
         <is>
           <t>95%</t>
         </is>
@@ -2146,12 +2149,12 @@
           <t>resume_Staff_Engineer-_Full_Stack_MER_Forbes_Advisor_132815.docx</t>
         </is>
       </c>
-      <c r="J28" s="58" t="inlineStr">
-        <is>
-          <t>No (Base)</t>
-        </is>
-      </c>
-      <c r="K28" s="58" t="inlineStr">
+      <c r="J28" s="60" t="inlineStr">
+        <is>
+          <t>No (Base)</t>
+        </is>
+      </c>
+      <c r="K28" s="60" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
@@ -2329,12 +2332,12 @@
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
-      <c r="A32" s="58" t="inlineStr">
-        <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="B32" s="58" t="inlineStr">
+      <c r="A32" s="60" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B32" s="60" t="inlineStr">
         <is>
           <t>4430692500</t>
         </is>
@@ -2359,7 +2362,7 @@
           <t>https://uk.linkedin.com/jobs/view/frontend-developer-at-haystack-4430692500</t>
         </is>
       </c>
-      <c r="G32" s="58" t="inlineStr">
+      <c r="G32" s="60" t="inlineStr">
         <is>
           <t>90%</t>
         </is>
@@ -2374,24 +2377,24 @@
           <t>resume_Frontend_Developer_Haystack_132900.docx</t>
         </is>
       </c>
-      <c r="J32" s="58" t="inlineStr">
-        <is>
-          <t>No (Base)</t>
-        </is>
-      </c>
-      <c r="K32" s="58" t="inlineStr">
+      <c r="J32" s="60" t="inlineStr">
+        <is>
+          <t>No (Base)</t>
+        </is>
+      </c>
+      <c r="K32" s="60" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1">
-      <c r="A33" s="58" t="inlineStr">
-        <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="B33" s="58" t="inlineStr">
+      <c r="A33" s="60" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B33" s="60" t="inlineStr">
         <is>
           <t>4433485213</t>
         </is>
@@ -2416,7 +2419,7 @@
           <t>https://in.linkedin.com/jobs/view/reactjs-developer-at-infosys-4433485213</t>
         </is>
       </c>
-      <c r="G33" s="58" t="inlineStr">
+      <c r="G33" s="60" t="inlineStr">
         <is>
           <t>90%</t>
         </is>
@@ -2431,12 +2434,12 @@
           <t>resume_ReactJS_developer_Infosys_132910.docx</t>
         </is>
       </c>
-      <c r="J33" s="58" t="inlineStr">
-        <is>
-          <t>No (Base)</t>
-        </is>
-      </c>
-      <c r="K33" s="58" t="inlineStr">
+      <c r="J33" s="60" t="inlineStr">
+        <is>
+          <t>No (Base)</t>
+        </is>
+      </c>
+      <c r="K33" s="60" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
@@ -2450,12 +2453,12 @@
       </c>
     </row>
     <row r="35" ht="18" customHeight="1">
-      <c r="A35" s="58" t="inlineStr">
-        <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="B35" s="58" t="inlineStr">
+      <c r="A35" s="60" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B35" s="60" t="inlineStr">
         <is>
           <t>4411903152</t>
         </is>
@@ -2480,7 +2483,7 @@
           <t>https://uk.linkedin.com/jobs/view/junior-full-stack-developer-at-inizio-engage-xd-4411903152</t>
         </is>
       </c>
-      <c r="G35" s="58" t="inlineStr">
+      <c r="G35" s="60" t="inlineStr">
         <is>
           <t>95%</t>
         </is>
@@ -2495,12 +2498,12 @@
           <t>resume_Junior_Full-Stack_Developer_Inizio_Engage_XD_133444.docx</t>
         </is>
       </c>
-      <c r="J35" s="58" t="inlineStr">
-        <is>
-          <t>No (Base)</t>
-        </is>
-      </c>
-      <c r="K35" s="58" t="inlineStr">
+      <c r="J35" s="60" t="inlineStr">
+        <is>
+          <t>No (Base)</t>
+        </is>
+      </c>
+      <c r="K35" s="60" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
@@ -2514,12 +2517,12 @@
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
-      <c r="A37" s="58" t="inlineStr">
-        <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="B37" s="58" t="inlineStr">
+      <c r="A37" s="60" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B37" s="60" t="inlineStr">
         <is>
           <t>4433469323</t>
         </is>
@@ -2544,7 +2547,7 @@
           <t>https://np.linkedin.com/jobs/view/software-engineer-at-tech-nirvana-4433469323</t>
         </is>
       </c>
-      <c r="G37" s="58" t="inlineStr">
+      <c r="G37" s="60" t="inlineStr">
         <is>
           <t>95%</t>
         </is>
@@ -2559,24 +2562,24 @@
           <t>resume_Software_Engineer_Tech_Nirvana_133917.docx</t>
         </is>
       </c>
-      <c r="J37" s="58" t="inlineStr">
-        <is>
-          <t>No (Base)</t>
-        </is>
-      </c>
-      <c r="K37" s="58" t="inlineStr">
+      <c r="J37" s="60" t="inlineStr">
+        <is>
+          <t>No (Base)</t>
+        </is>
+      </c>
+      <c r="K37" s="60" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
-      <c r="A38" s="58" t="inlineStr">
-        <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="B38" s="58" t="inlineStr">
+      <c r="A38" s="60" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B38" s="60" t="inlineStr">
         <is>
           <t>4432690812</t>
         </is>
@@ -2601,7 +2604,7 @@
           <t>https://bd.linkedin.com/jobs/view/we%E2%80%99re-looking-for-mern-stack-developers%21-at-impala-intech-software-development-agency-4432690812</t>
         </is>
       </c>
-      <c r="G38" s="58" t="inlineStr">
+      <c r="G38" s="60" t="inlineStr">
         <is>
           <t>100%</t>
         </is>
@@ -2616,12 +2619,12 @@
           <t>resume_Were_Looking_For_MERN_Stack_De_Impala_Intech_-_So_133928.docx</t>
         </is>
       </c>
-      <c r="J38" s="58" t="inlineStr">
-        <is>
-          <t>No (Base)</t>
-        </is>
-      </c>
-      <c r="K38" s="58" t="inlineStr">
+      <c r="J38" s="60" t="inlineStr">
+        <is>
+          <t>No (Base)</t>
+        </is>
+      </c>
+      <c r="K38" s="60" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
@@ -2799,12 +2802,12 @@
       </c>
     </row>
     <row r="42" ht="18" customHeight="1">
-      <c r="A42" s="58" t="inlineStr">
-        <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="B42" s="58" t="inlineStr">
+      <c r="A42" s="60" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B42" s="60" t="inlineStr">
         <is>
           <t>4393032766</t>
         </is>
@@ -2829,7 +2832,7 @@
           <t>https://in.linkedin.com/jobs/view/react-js-developer-at-infosys-4393032766</t>
         </is>
       </c>
-      <c r="G42" s="58" t="inlineStr">
+      <c r="G42" s="60" t="inlineStr">
         <is>
           <t>90%</t>
         </is>
@@ -2844,24 +2847,24 @@
           <t>resume_React_JS_Developer_Infosys_134020.docx</t>
         </is>
       </c>
-      <c r="J42" s="58" t="inlineStr">
-        <is>
-          <t>No (Base)</t>
-        </is>
-      </c>
-      <c r="K42" s="58" t="inlineStr">
+      <c r="J42" s="60" t="inlineStr">
+        <is>
+          <t>No (Base)</t>
+        </is>
+      </c>
+      <c r="K42" s="60" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
       </c>
     </row>
     <row r="43" ht="18" customHeight="1">
-      <c r="A43" s="58" t="inlineStr">
-        <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="B43" s="58" t="inlineStr">
+      <c r="A43" s="60" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B43" s="60" t="inlineStr">
         <is>
           <t>4433313819</t>
         </is>
@@ -2886,7 +2889,7 @@
           <t>https://ca.linkedin.com/jobs/view/react-developer-at-altimetrik-4433313819</t>
         </is>
       </c>
-      <c r="G43" s="58" t="inlineStr">
+      <c r="G43" s="60" t="inlineStr">
         <is>
           <t>95%</t>
         </is>
@@ -2901,12 +2904,12 @@
           <t>resume_React_Developer_Altimetrik_134033.docx</t>
         </is>
       </c>
-      <c r="J43" s="58" t="inlineStr">
-        <is>
-          <t>No (Base)</t>
-        </is>
-      </c>
-      <c r="K43" s="58" t="inlineStr">
+      <c r="J43" s="60" t="inlineStr">
+        <is>
+          <t>No (Base)</t>
+        </is>
+      </c>
+      <c r="K43" s="60" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
@@ -2970,12 +2973,12 @@
       </c>
     </row>
     <row r="45" ht="18" customHeight="1">
-      <c r="A45" s="58" t="inlineStr">
-        <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="B45" s="58" t="inlineStr">
+      <c r="A45" s="60" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B45" s="60" t="inlineStr">
         <is>
           <t>4429984849</t>
         </is>
@@ -3000,7 +3003,7 @@
           <t>https://ca.linkedin.com/jobs/view/reactjs-developer-at-covetus-4429984849</t>
         </is>
       </c>
-      <c r="G45" s="58" t="inlineStr">
+      <c r="G45" s="60" t="inlineStr">
         <is>
           <t>95%</t>
         </is>
@@ -3015,24 +3018,24 @@
           <t>resume_ReactJS_Developer_Covetus_134059.docx</t>
         </is>
       </c>
-      <c r="J45" s="58" t="inlineStr">
-        <is>
-          <t>No (Base)</t>
-        </is>
-      </c>
-      <c r="K45" s="58" t="inlineStr">
+      <c r="J45" s="60" t="inlineStr">
+        <is>
+          <t>No (Base)</t>
+        </is>
+      </c>
+      <c r="K45" s="60" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
       </c>
     </row>
     <row r="46" ht="18" customHeight="1">
-      <c r="A46" s="58" t="inlineStr">
-        <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="B46" s="58" t="inlineStr">
+      <c r="A46" s="60" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B46" s="60" t="inlineStr">
         <is>
           <t>4434104517</t>
         </is>
@@ -3057,7 +3060,7 @@
           <t>https://ca.linkedin.com/jobs/view/frontend-developer-react-at-newnovation-solutions-4434104517</t>
         </is>
       </c>
-      <c r="G46" s="58" t="inlineStr">
+      <c r="G46" s="60" t="inlineStr">
         <is>
           <t>95%</t>
         </is>
@@ -3072,24 +3075,24 @@
           <t>resume_Frontend_Developer-React_Newnovation_Soluti_134111.docx</t>
         </is>
       </c>
-      <c r="J46" s="58" t="inlineStr">
-        <is>
-          <t>No (Base)</t>
-        </is>
-      </c>
-      <c r="K46" s="58" t="inlineStr">
+      <c r="J46" s="60" t="inlineStr">
+        <is>
+          <t>No (Base)</t>
+        </is>
+      </c>
+      <c r="K46" s="60" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
       </c>
     </row>
     <row r="47" ht="18" customHeight="1">
-      <c r="A47" s="58" t="inlineStr">
-        <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="B47" s="58" t="inlineStr">
+      <c r="A47" s="60" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B47" s="60" t="inlineStr">
         <is>
           <t>4432641330</t>
         </is>
@@ -3114,7 +3117,7 @@
           <t>https://id.linkedin.com/jobs/view/junior-web-developer-frontend-backend-at-nordia-digital-4432641330</t>
         </is>
       </c>
-      <c r="G47" s="58" t="inlineStr">
+      <c r="G47" s="60" t="inlineStr">
         <is>
           <t>95%</t>
         </is>
@@ -3129,12 +3132,12 @@
           <t>resume_Junior_Web_Developer_FrontendB_Nordia_Digital_134123.docx</t>
         </is>
       </c>
-      <c r="J47" s="58" t="inlineStr">
-        <is>
-          <t>No (Base)</t>
-        </is>
-      </c>
-      <c r="K47" s="58" t="inlineStr">
+      <c r="J47" s="60" t="inlineStr">
+        <is>
+          <t>No (Base)</t>
+        </is>
+      </c>
+      <c r="K47" s="60" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
@@ -3212,12 +3215,12 @@
       </c>
     </row>
     <row r="51" ht="18" customHeight="1">
-      <c r="A51" s="58" t="inlineStr">
-        <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="B51" s="58" t="inlineStr">
+      <c r="A51" s="60" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B51" s="60" t="inlineStr">
         <is>
           <t>9999999</t>
         </is>
@@ -3242,7 +3245,7 @@
           <t>https://linkedin.com</t>
         </is>
       </c>
-      <c r="G51" s="58" t="inlineStr">
+      <c r="G51" s="60" t="inlineStr">
         <is>
           <t>98%</t>
         </is>
@@ -3257,12 +3260,12 @@
           <t>resume_React_Developer_Perfect_Layout.pdf</t>
         </is>
       </c>
-      <c r="J51" s="58" t="inlineStr">
+      <c r="J51" s="60" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="K51" s="58" t="inlineStr">
+      <c r="K51" s="60" t="inlineStr">
         <is>
           <t>Verified</t>
         </is>
@@ -3497,12 +3500,12 @@
       </c>
     </row>
     <row r="56" ht="18" customHeight="1">
-      <c r="A56" s="58" t="inlineStr">
-        <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="B56" s="58" t="inlineStr">
+      <c r="A56" s="60" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B56" s="60" t="inlineStr">
         <is>
           <t>4433308436</t>
         </is>
@@ -3527,7 +3530,7 @@
           <t>https://uk.linkedin.com/jobs/view/javascript-developer-at-socode-recruitment-4433308436</t>
         </is>
       </c>
-      <c r="G56" s="58" t="inlineStr">
+      <c r="G56" s="60" t="inlineStr">
         <is>
           <t>100%</t>
         </is>
@@ -3542,12 +3545,12 @@
           <t>resume_Javascript_Developer_SoCode_Recruitment_150742.docx</t>
         </is>
       </c>
-      <c r="J56" s="58" t="inlineStr">
-        <is>
-          <t>No (Base)</t>
-        </is>
-      </c>
-      <c r="K56" s="58" t="inlineStr">
+      <c r="J56" s="60" t="inlineStr">
+        <is>
+          <t>No (Base)</t>
+        </is>
+      </c>
+      <c r="K56" s="60" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
@@ -3611,12 +3614,12 @@
       </c>
     </row>
     <row r="58" ht="18" customHeight="1">
-      <c r="A58" s="58" t="inlineStr">
-        <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="B58" s="58" t="inlineStr">
+      <c r="A58" s="60" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B58" s="60" t="inlineStr">
         <is>
           <t>4433350368</t>
         </is>
@@ -3641,7 +3644,7 @@
           <t>https://uk.linkedin.com/jobs/view/web-software-engineer-at-virgin-active-4433350368</t>
         </is>
       </c>
-      <c r="G58" s="58" t="inlineStr">
+      <c r="G58" s="60" t="inlineStr">
         <is>
           <t>90%</t>
         </is>
@@ -3656,12 +3659,12 @@
           <t>resume_Web_Software_Engineer_Virgin_Active_150804.docx</t>
         </is>
       </c>
-      <c r="J58" s="58" t="inlineStr">
-        <is>
-          <t>No (Base)</t>
-        </is>
-      </c>
-      <c r="K58" s="58" t="inlineStr">
+      <c r="J58" s="60" t="inlineStr">
+        <is>
+          <t>No (Base)</t>
+        </is>
+      </c>
+      <c r="K58" s="60" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
@@ -3675,12 +3678,12 @@
       </c>
     </row>
     <row r="60" ht="18" customHeight="1">
-      <c r="A60" s="58" t="inlineStr">
-        <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="B60" s="58" t="inlineStr">
+      <c r="A60" s="60" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B60" s="60" t="inlineStr">
         <is>
           <t>8888888</t>
         </is>
@@ -3705,7 +3708,7 @@
           <t>https://linkedin.com</t>
         </is>
       </c>
-      <c r="G60" s="58" t="inlineStr">
+      <c r="G60" s="60" t="inlineStr">
         <is>
           <t>99%</t>
         </is>
@@ -3720,24 +3723,24 @@
           <t>resume_Full_Stack_Executive_Spacing.pdf</t>
         </is>
       </c>
-      <c r="J60" s="58" t="inlineStr">
+      <c r="J60" s="60" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="K60" s="58" t="inlineStr">
+      <c r="K60" s="60" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
       </c>
     </row>
     <row r="61" ht="18" customHeight="1">
-      <c r="A61" s="59" t="inlineStr">
-        <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="B61" s="59" t="inlineStr">
+      <c r="A61" s="60" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B61" s="60" t="inlineStr">
         <is>
           <t>7777777</t>
         </is>
@@ -3762,7 +3765,7 @@
           <t>https://linkedin.com</t>
         </is>
       </c>
-      <c r="G61" s="59" t="inlineStr">
+      <c r="G61" s="60" t="inlineStr">
         <is>
           <t>100%</t>
         </is>
@@ -3777,25 +3780,90 @@
           <t>resume_Full_Stack_FoodFlow_1Page.pdf</t>
         </is>
       </c>
-      <c r="J61" s="59" t="inlineStr">
+      <c r="J61" s="60" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="K61" s="59" t="inlineStr">
+      <c r="K61" s="60" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
       </c>
     </row>
+    <row r="62" ht="18" customHeight="1">
+      <c r="A62" s="60" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B62" s="60" t="inlineStr">
+        <is>
+          <t>4433462994</t>
+        </is>
+      </c>
+      <c r="C62" s="3" t="inlineStr">
+        <is>
+          <t>Reactjs Developer</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="inlineStr">
+        <is>
+          <t>Infosys</t>
+        </is>
+      </c>
+      <c r="E62" s="3" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="F62" s="4" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/jobs/view/reactjs-developer-at-infosys-4433462994</t>
+        </is>
+      </c>
+      <c r="G62" s="60" t="inlineStr">
+        <is>
+          <t>95%</t>
+        </is>
+      </c>
+      <c r="H62" s="3" t="inlineStr">
+        <is>
+          <t>Strong Reactjs skills and relevant experience</t>
+        </is>
+      </c>
+      <c r="I62" s="4" t="inlineStr">
+        <is>
+          <t>resume_Reactjs_Developer_Infosys_153704.docx</t>
+        </is>
+      </c>
+      <c r="J62" s="60" t="inlineStr">
+        <is>
+          <t>No (Base)</t>
+        </is>
+      </c>
+      <c r="K62" s="60" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="20" t="inlineStr">
+        <is>
+          <t>--- Run Summary (2026-06-29 15:37 UTC) | Scraped: 18 | New: 1 | Passed: 1 | CVs: 1 | Errors: 0 ---</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="8">
     <mergeCell ref="A34:K34"/>
     <mergeCell ref="A50:K50"/>
     <mergeCell ref="A18:K18"/>
     <mergeCell ref="A59:K59"/>
     <mergeCell ref="A16:K16"/>
     <mergeCell ref="A49:K49"/>
+    <mergeCell ref="A63:K63"/>
     <mergeCell ref="A36:K36"/>
   </mergeCells>
   <hyperlinks>
@@ -3904,6 +3972,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I60" r:id="rId103"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F61" r:id="rId104"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I61" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F62" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I62" r:id="rId107"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>